<commit_message>
KPI actualizado 2026-08-28 14:35 UTC
</commit_message>
<xml_diff>
--- a/data/50001592 - VITA EXPRESS INC (Venezuela).xlsx
+++ b/data/50001592 - VITA EXPRESS INC (Venezuela).xlsx
@@ -4478,7 +4478,7 @@
       </c>
       <c r="C49" s="10"/>
       <c r="D49" s="9">
-        <v>46240.58279298611</v>
+        <v>46262.606391203706</v>
       </c>
       <c r="E49" s="10" t="s">
         <v>167</v>
@@ -4523,9 +4523,11 @@
       <c r="B50" s="5">
         <v>46239.574202800926</v>
       </c>
-      <c r="C50" s="6"/>
+      <c r="C50" s="5">
+        <v>46262.60637799768</v>
+      </c>
       <c r="D50" s="5">
-        <v>46262.17148158565</v>
+        <v>46262.606404039354</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>170</v>
@@ -4573,10 +4575,10 @@
         <v>174</v>
       </c>
       <c r="T50" s="6">
-        <v>0</v>
-      </c>
-      <c r="U50" s="12" t="s">
-        <v>49</v>
+        <v>1</v>
+      </c>
+      <c r="U50" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
@@ -4588,7 +4590,7 @@
       </c>
       <c r="C51" s="10"/>
       <c r="D51" s="9">
-        <v>46251.97138391204</v>
+        <v>46262.60639164352</v>
       </c>
       <c r="E51" s="10" t="s">
         <v>176</v>

</xml_diff>